<commit_message>
Update description of features.xlsx
</commit_message>
<xml_diff>
--- a/description of features.xlsx
+++ b/description of features.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="21">
   <si>
     <t xml:space="preserve">Название признака </t>
   </si>
@@ -64,6 +64,24 @@
   </si>
   <si>
     <t>Признаки по видам экономической деятельности (приставка _s - sector)</t>
+  </si>
+  <si>
+    <t>Численность работников, выполнявших научные исследования и разработки</t>
+  </si>
+  <si>
+    <t>researchers_s</t>
+  </si>
+  <si>
+    <t>2017-2024</t>
+  </si>
+  <si>
+    <t>11_ОКВЭД2_публ.xlsx</t>
+  </si>
+  <si>
+    <t>1_2 ОКВЭД2_публ.xlsx</t>
+  </si>
+  <si>
+    <t>Исходник-форма (росстат)</t>
   </si>
 </sst>
 </file>
@@ -412,7 +430,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25.85546875" customWidth="1"/>
@@ -421,14 +439,15 @@
     <col min="4" max="4" width="19.140625" customWidth="1"/>
     <col min="5" max="5" width="21.5703125" customWidth="1"/>
     <col min="6" max="6" width="25.28515625" customWidth="1"/>
+    <col min="7" max="7" width="26.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B1" s="5" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -447,8 +466,11 @@
       <c r="F2" s="1" t="s">
         <v>9</v>
       </c>
+      <c r="G2" s="1" t="s">
+        <v>20</v>
+      </c>
     </row>
-    <row r="3" spans="1:6" ht="45" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>4</v>
       </c>
@@ -467,8 +489,11 @@
       <c r="F3" s="2" t="s">
         <v>10</v>
       </c>
+      <c r="G3" s="2" t="s">
+        <v>19</v>
+      </c>
     </row>
-    <row r="4" spans="1:6" ht="60" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" ht="60" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>12</v>
       </c>
@@ -486,6 +511,32 @@
       </c>
       <c r="F4" s="2" t="s">
         <v>10</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="E5" s="2">
+        <v>1814</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>18</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
AI and Skvoz-tech costs in regions
</commit_message>
<xml_diff>
--- a/description of features.xlsx
+++ b/description of features.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="76">
   <si>
     <t xml:space="preserve">Название признака </t>
   </si>
@@ -233,6 +233,21 @@
   </si>
   <si>
     <t>PCusage_r</t>
+  </si>
+  <si>
+    <t>AIcosts_r</t>
+  </si>
+  <si>
+    <t>ITcosts_r</t>
+  </si>
+  <si>
+    <t>skvozcosts_r</t>
+  </si>
+  <si>
+    <t>trainingcosts_r</t>
+  </si>
+  <si>
+    <t>47_ОКАТО.xlsx</t>
   </si>
 </sst>
 </file>
@@ -1158,7 +1173,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G8"/>
+  <dimension ref="A1:G16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="36.140625" customWidth="1"/>
@@ -1324,6 +1339,105 @@
         <v>64</v>
       </c>
     </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="B12" s="3"/>
+      <c r="C12" s="3"/>
+      <c r="D12" s="3"/>
+      <c r="E12" s="3"/>
+      <c r="F12" s="3"/>
+      <c r="G12" s="3"/>
+    </row>
+    <row r="13" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A13" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="B13" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="D13" s="4">
+        <v>2024</v>
+      </c>
+      <c r="E13" s="4">
+        <v>94</v>
+      </c>
+      <c r="F13" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="G13" s="4" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A14" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="B14" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E14" s="4"/>
+      <c r="F14" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="G14" s="4" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A15" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="B15" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="D15" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="E15" s="4">
+        <v>470</v>
+      </c>
+      <c r="F15" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="G15" s="4" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+      <c r="A16" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="B16" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="D16" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E16" s="4"/>
+      <c r="F16" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="G16" s="4" t="s">
+        <v>75</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
IT costs in regions
</commit_message>
<xml_diff>
--- a/description of features.xlsx
+++ b/description of features.xlsx
@@ -1386,7 +1386,9 @@
       <c r="D14" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="E14" s="4"/>
+      <c r="E14" s="4">
+        <v>846</v>
+      </c>
       <c r="F14" s="4" t="s">
         <v>63</v>
       </c>
@@ -1430,7 +1432,9 @@
       <c r="D16" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="E16" s="4"/>
+      <c r="E16" s="4">
+        <v>846</v>
+      </c>
       <c r="F16" s="4" t="s">
         <v>63</v>
       </c>

</xml_diff>

<commit_message>
upd. description of features
</commit_message>
<xml_diff>
--- a/description of features.xlsx
+++ b/description of features.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
   </bookViews>
   <sheets>
     <sheet name="По отраслям" sheetId="1" r:id="rId1"/>
@@ -1225,7 +1225,7 @@
         <v>27</v>
       </c>
       <c r="E23" s="20">
-        <v>171</v>
+        <v>513</v>
       </c>
       <c r="F23" s="20" t="s">
         <v>10</v>

</xml_diff>